<commit_message>
Updated Cecidomyiidae taxonomy and traits source file
</commit_message>
<xml_diff>
--- a/source_data/Cecidomyiidae_taxonomy_traits.xlsx
+++ b/source_data/Cecidomyiidae_taxonomy_traits.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EFFAACA-F41B-5141-A360-1EFB262FA36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD2C0D5-8431-E440-BC3F-1408DF7D1511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="27840" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="27840" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw data" sheetId="1" r:id="rId1"/>
-    <sheet name="Trait data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621" concurrentCalc="0"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="28">
   <si>
     <t>Insecta</t>
   </si>
@@ -146,34 +145,7 @@
     <t>Clade</t>
   </si>
   <si>
-    <t>Niche</t>
-  </si>
-  <si>
-    <t>Habitat</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>Lasiopteridi</t>
-  </si>
-  <si>
-    <t>Lestodiplosini</t>
-  </si>
-  <si>
-    <t>Cecidomyiidi</t>
-  </si>
-  <si>
-    <t>Stomatosematidi</t>
-  </si>
-  <si>
     <t>Subfamily</t>
-  </si>
-  <si>
-    <t>Aphidoletini</t>
-  </si>
-  <si>
-    <t>Predator</t>
   </si>
   <si>
     <t>Phytophage</t>
@@ -249,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -276,12 +248,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -300,9 +266,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -340,7 +306,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -446,7 +412,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -588,7 +554,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -618,7 +584,7 @@
         <v>15</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>24</v>
@@ -682,13 +648,13 @@
         <v>8</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>7</v>
@@ -835,176 +801,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB226CCB-A10B-A549-8C0D-6D70F7C68B48}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="18.5" customWidth="1"/>
-    <col min="3" max="4" width="12.1640625" style="11" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>